<commit_message>
update new inventory files
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_bulgaria_transformation_nov_27.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_bulgaria_transformation_nov_27.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/sisepuede_modeling/ssp_bulgaria/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F96755F-917C-3045-8237-F11BE131DD31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3089F1FC-A942-9541-9AF1-A62ACCFAA907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="35360" windowHeight="26860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="447">
   <si>
     <t>subsector</t>
   </si>
@@ -1448,9 +1448,6 @@
   </si>
   <si>
     <t>They mention wastewater treatment related to industrial processes.</t>
-  </si>
-  <si>
-    <t>%</t>
   </si>
 </sst>
 </file>
@@ -2094,16 +2091,16 @@
   <cols>
     <col min="1" max="2" width="13.1640625" style="4" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="43.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.6640625" style="4" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="31.6640625" style="4" customWidth="1"/>
     <col min="5" max="5" width="62.5" style="4" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="33.1640625" style="4" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="71.33203125" style="4" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="30.5" style="4" customWidth="1"/>
     <col min="8" max="8" width="39.33203125" style="4" customWidth="1"/>
     <col min="9" max="9" width="13.83203125" style="4" customWidth="1"/>
     <col min="10" max="10" width="14.1640625" style="4" customWidth="1"/>
     <col min="11" max="12" width="35" style="4" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="31.5" style="36" customWidth="1"/>
-    <col min="14" max="14" width="19.83203125" style="35" customWidth="1"/>
+    <col min="13" max="13" width="31.5" style="36" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="19.83203125" style="35" hidden="1" customWidth="1"/>
     <col min="15" max="16" width="20.5" style="37" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="13.5" style="38" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="13.5" style="37" bestFit="1" customWidth="1"/>
@@ -4700,8 +4697,8 @@
       <c r="O57" s="16">
         <v>1</v>
       </c>
-      <c r="P57" s="16" t="s">
-        <v>447</v>
+      <c r="P57" s="16">
+        <v>1</v>
       </c>
       <c r="Q57" s="10"/>
       <c r="R57" s="11"/>
@@ -4785,8 +4782,12 @@
       <c r="H59" s="12" t="s">
         <v>442</v>
       </c>
-      <c r="I59" s="26"/>
-      <c r="J59" s="26"/>
+      <c r="I59" s="26">
+        <v>1</v>
+      </c>
+      <c r="J59" s="26">
+        <v>1</v>
+      </c>
       <c r="K59" s="44"/>
       <c r="L59" s="44"/>
       <c r="M59" s="15">
@@ -4832,8 +4833,12 @@
       <c r="H60" s="12" t="s">
         <v>442</v>
       </c>
-      <c r="I60" s="12"/>
-      <c r="J60" s="12"/>
+      <c r="I60" s="12">
+        <v>1</v>
+      </c>
+      <c r="J60" s="12">
+        <v>1</v>
+      </c>
       <c r="K60" s="12"/>
       <c r="L60" s="12"/>
       <c r="M60" s="15">

</xml_diff>